<commit_message>
Upload latest bio-printing files
</commit_message>
<xml_diff>
--- a/database/data/raw/metadata/bioprint_metadata_template_v2.xlsx
+++ b/database/data/raw/metadata/bioprint_metadata_template_v2.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="24">
   <si>
     <t>image_path</t>
   </si>
@@ -122,6 +122,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
       <t>补速度</t>
     </r>
     <r>
@@ -172,6 +178,12 @@
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="宋体"/>
+        <charset val="134"/>
+      </rPr>
       <t>修改高度为</t>
     </r>
     <r>
@@ -186,6 +198,12 @@
   </si>
   <si>
     <t>挤出速度再小无法成型，高度是否还能增大，放大挤出速度？</t>
+  </si>
+  <si>
+    <t>忘记调速度了。。。</t>
+  </si>
+  <si>
+    <t>重新补上</t>
   </si>
 </sst>
 </file>
@@ -2962,968 +2980,1852 @@
     </row>
     <row r="74" spans="1:9">
       <c r="A74" s="3"/>
-      <c r="B74" s="8"/>
-      <c r="C74" s="8"/>
-      <c r="D74" s="8"/>
-      <c r="E74" s="8"/>
-      <c r="F74" s="8"/>
+      <c r="B74" s="8">
+        <v>73</v>
+      </c>
+      <c r="C74" s="8">
+        <v>15</v>
+      </c>
+      <c r="D74" s="8">
+        <v>8</v>
+      </c>
+      <c r="E74" s="8">
+        <v>3</v>
+      </c>
+      <c r="F74" s="8">
+        <v>5</v>
+      </c>
       <c r="G74" s="8"/>
       <c r="H74" s="3"/>
       <c r="I74" s="3"/>
     </row>
     <row r="75" spans="1:9">
       <c r="A75" s="3"/>
-      <c r="B75" s="8"/>
-      <c r="C75" s="8"/>
-      <c r="D75" s="8"/>
-      <c r="E75" s="8"/>
-      <c r="F75" s="8"/>
+      <c r="B75" s="8">
+        <v>74</v>
+      </c>
+      <c r="C75" s="8">
+        <v>15</v>
+      </c>
+      <c r="D75" s="8">
+        <v>7</v>
+      </c>
+      <c r="E75" s="8">
+        <v>3</v>
+      </c>
+      <c r="F75" s="8">
+        <v>5</v>
+      </c>
       <c r="G75" s="8"/>
       <c r="H75" s="3"/>
       <c r="I75" s="3"/>
     </row>
     <row r="76" spans="1:9">
       <c r="A76" s="3"/>
-      <c r="B76" s="8"/>
-      <c r="C76" s="8"/>
-      <c r="D76" s="8"/>
-      <c r="E76" s="8"/>
-      <c r="F76" s="8"/>
+      <c r="B76" s="8">
+        <v>75</v>
+      </c>
+      <c r="C76" s="8">
+        <v>15</v>
+      </c>
+      <c r="D76" s="8">
+        <v>6</v>
+      </c>
+      <c r="E76" s="8">
+        <v>3</v>
+      </c>
+      <c r="F76" s="8">
+        <v>5</v>
+      </c>
       <c r="G76" s="8"/>
       <c r="H76" s="3"/>
       <c r="I76" s="3"/>
     </row>
     <row r="77" spans="1:9">
       <c r="A77" s="3"/>
-      <c r="B77" s="8"/>
-      <c r="C77" s="8"/>
-      <c r="D77" s="8"/>
-      <c r="E77" s="8"/>
-      <c r="F77" s="8"/>
+      <c r="B77" s="8">
+        <v>76</v>
+      </c>
+      <c r="C77" s="8">
+        <v>15</v>
+      </c>
+      <c r="D77" s="8">
+        <v>5</v>
+      </c>
+      <c r="E77" s="8">
+        <v>3</v>
+      </c>
+      <c r="F77" s="8">
+        <v>5</v>
+      </c>
       <c r="G77" s="8"/>
       <c r="H77" s="3"/>
       <c r="I77" s="3"/>
     </row>
     <row r="78" spans="1:9">
       <c r="A78" s="3"/>
-      <c r="B78" s="8"/>
-      <c r="C78" s="8"/>
-      <c r="D78" s="8"/>
-      <c r="E78" s="8"/>
-      <c r="F78" s="8"/>
+      <c r="B78" s="8">
+        <v>77</v>
+      </c>
+      <c r="C78" s="8">
+        <v>15</v>
+      </c>
+      <c r="D78" s="8">
+        <v>4</v>
+      </c>
+      <c r="E78" s="8">
+        <v>3</v>
+      </c>
+      <c r="F78" s="8">
+        <v>5</v>
+      </c>
       <c r="G78" s="8"/>
       <c r="H78" s="3"/>
       <c r="I78" s="3"/>
     </row>
     <row r="79" spans="1:9">
       <c r="A79" s="3"/>
-      <c r="B79" s="8"/>
-      <c r="C79" s="8"/>
-      <c r="D79" s="8"/>
-      <c r="E79" s="8"/>
-      <c r="F79" s="8"/>
+      <c r="B79" s="8">
+        <v>78</v>
+      </c>
+      <c r="C79" s="8">
+        <v>15</v>
+      </c>
+      <c r="D79" s="8">
+        <v>3</v>
+      </c>
+      <c r="E79" s="8">
+        <v>3</v>
+      </c>
+      <c r="F79" s="8">
+        <v>5</v>
+      </c>
       <c r="G79" s="8"/>
       <c r="H79" s="3"/>
       <c r="I79" s="3"/>
     </row>
     <row r="80" spans="1:9">
       <c r="A80" s="3"/>
-      <c r="B80" s="8"/>
-      <c r="C80" s="8"/>
-      <c r="D80" s="8"/>
-      <c r="E80" s="8"/>
-      <c r="F80" s="8"/>
+      <c r="B80" s="8">
+        <v>79</v>
+      </c>
+      <c r="C80" s="8">
+        <v>15</v>
+      </c>
+      <c r="D80" s="8">
+        <v>2</v>
+      </c>
+      <c r="E80" s="8">
+        <v>3</v>
+      </c>
+      <c r="F80" s="8">
+        <v>5</v>
+      </c>
       <c r="G80" s="8"/>
       <c r="H80" s="3"/>
       <c r="I80" s="3"/>
     </row>
     <row r="81" spans="1:9">
       <c r="A81" s="3"/>
-      <c r="B81" s="8"/>
-      <c r="C81" s="8"/>
-      <c r="D81" s="8"/>
-      <c r="E81" s="8"/>
-      <c r="F81" s="8"/>
+      <c r="B81" s="8">
+        <v>80</v>
+      </c>
+      <c r="C81" s="8">
+        <v>20</v>
+      </c>
+      <c r="D81" s="8">
+        <v>6</v>
+      </c>
+      <c r="E81" s="8">
+        <v>3</v>
+      </c>
+      <c r="F81" s="8">
+        <v>3.5</v>
+      </c>
       <c r="G81" s="8"/>
       <c r="H81" s="3"/>
       <c r="I81" s="3"/>
     </row>
     <row r="82" spans="1:9">
       <c r="A82" s="3"/>
-      <c r="B82" s="8"/>
-      <c r="C82" s="8"/>
-      <c r="D82" s="8"/>
-      <c r="E82" s="8"/>
-      <c r="F82" s="8"/>
+      <c r="B82" s="8">
+        <v>81</v>
+      </c>
+      <c r="C82" s="8">
+        <v>20</v>
+      </c>
+      <c r="D82" s="8">
+        <v>7</v>
+      </c>
+      <c r="E82" s="8">
+        <v>3</v>
+      </c>
+      <c r="F82" s="8">
+        <v>3.5</v>
+      </c>
       <c r="G82" s="8"/>
       <c r="H82" s="3"/>
       <c r="I82" s="3"/>
     </row>
     <row r="83" spans="1:9">
       <c r="A83" s="3"/>
-      <c r="B83" s="8"/>
-      <c r="C83" s="8"/>
-      <c r="D83" s="8"/>
-      <c r="E83" s="8"/>
-      <c r="F83" s="8"/>
+      <c r="B83" s="8">
+        <v>82</v>
+      </c>
+      <c r="C83" s="8">
+        <v>20</v>
+      </c>
+      <c r="D83" s="8">
+        <v>8</v>
+      </c>
+      <c r="E83" s="8">
+        <v>3</v>
+      </c>
+      <c r="F83" s="8">
+        <v>3.5</v>
+      </c>
       <c r="G83" s="8"/>
       <c r="H83" s="3"/>
       <c r="I83" s="3"/>
     </row>
     <row r="84" spans="1:9">
       <c r="A84" s="3"/>
-      <c r="B84" s="8"/>
-      <c r="C84" s="8"/>
-      <c r="D84" s="8"/>
-      <c r="E84" s="8"/>
-      <c r="F84" s="8"/>
+      <c r="B84" s="8">
+        <v>83</v>
+      </c>
+      <c r="C84" s="8">
+        <v>20</v>
+      </c>
+      <c r="D84" s="8">
+        <v>9</v>
+      </c>
+      <c r="E84" s="8">
+        <v>3</v>
+      </c>
+      <c r="F84" s="8">
+        <v>3.5</v>
+      </c>
       <c r="G84" s="8"/>
       <c r="H84" s="3"/>
       <c r="I84" s="3"/>
     </row>
     <row r="85" spans="1:9">
       <c r="A85" s="3"/>
-      <c r="B85" s="8"/>
-      <c r="C85" s="8"/>
-      <c r="D85" s="8"/>
-      <c r="E85" s="8"/>
-      <c r="F85" s="8"/>
+      <c r="B85" s="8">
+        <v>84</v>
+      </c>
+      <c r="C85" s="8">
+        <v>20</v>
+      </c>
+      <c r="D85" s="8">
+        <v>1</v>
+      </c>
+      <c r="E85" s="8">
+        <v>3</v>
+      </c>
+      <c r="F85" s="8">
+        <v>4</v>
+      </c>
       <c r="G85" s="8"/>
       <c r="H85" s="3"/>
       <c r="I85" s="3"/>
     </row>
     <row r="86" spans="1:9">
       <c r="A86" s="3"/>
-      <c r="B86" s="8"/>
-      <c r="C86" s="8"/>
-      <c r="D86" s="8"/>
-      <c r="E86" s="8"/>
-      <c r="F86" s="8"/>
+      <c r="B86" s="8">
+        <v>85</v>
+      </c>
+      <c r="C86" s="8">
+        <v>20</v>
+      </c>
+      <c r="D86" s="8">
+        <v>2</v>
+      </c>
+      <c r="E86" s="8">
+        <v>3</v>
+      </c>
+      <c r="F86" s="8">
+        <v>4</v>
+      </c>
       <c r="G86" s="8"/>
       <c r="H86" s="3"/>
       <c r="I86" s="3"/>
     </row>
     <row r="87" spans="1:9">
       <c r="A87" s="3"/>
-      <c r="B87" s="8"/>
-      <c r="C87" s="8"/>
-      <c r="D87" s="8"/>
-      <c r="E87" s="8"/>
-      <c r="F87" s="8"/>
+      <c r="B87" s="8">
+        <v>86</v>
+      </c>
+      <c r="C87" s="8">
+        <v>20</v>
+      </c>
+      <c r="D87" s="8">
+        <v>3</v>
+      </c>
+      <c r="E87" s="8">
+        <v>3</v>
+      </c>
+      <c r="F87" s="8">
+        <v>4</v>
+      </c>
       <c r="G87" s="8"/>
       <c r="H87" s="3"/>
       <c r="I87" s="3"/>
     </row>
     <row r="88" spans="1:9">
       <c r="A88" s="3"/>
-      <c r="B88" s="8"/>
-      <c r="C88" s="8"/>
-      <c r="D88" s="8"/>
-      <c r="E88" s="8"/>
-      <c r="F88" s="8"/>
+      <c r="B88" s="8">
+        <v>87</v>
+      </c>
+      <c r="C88" s="8">
+        <v>20</v>
+      </c>
+      <c r="D88" s="8">
+        <v>4</v>
+      </c>
+      <c r="E88" s="8">
+        <v>3</v>
+      </c>
+      <c r="F88" s="8">
+        <v>4</v>
+      </c>
       <c r="G88" s="8"/>
       <c r="H88" s="3"/>
       <c r="I88" s="3"/>
     </row>
     <row r="89" spans="1:9">
       <c r="A89" s="3"/>
-      <c r="B89" s="8"/>
-      <c r="C89" s="8"/>
-      <c r="D89" s="8"/>
-      <c r="E89" s="8"/>
-      <c r="F89" s="8"/>
+      <c r="B89" s="8">
+        <v>88</v>
+      </c>
+      <c r="C89" s="8">
+        <v>20</v>
+      </c>
+      <c r="D89" s="8">
+        <v>5</v>
+      </c>
+      <c r="E89" s="8">
+        <v>3</v>
+      </c>
+      <c r="F89" s="8">
+        <v>4</v>
+      </c>
       <c r="G89" s="8"/>
       <c r="H89" s="3"/>
       <c r="I89" s="3"/>
     </row>
     <row r="90" spans="1:9">
       <c r="A90" s="3"/>
-      <c r="B90" s="8"/>
-      <c r="C90" s="8"/>
-      <c r="D90" s="8"/>
-      <c r="E90" s="8"/>
-      <c r="F90" s="8"/>
+      <c r="B90" s="8">
+        <v>89</v>
+      </c>
+      <c r="C90" s="8">
+        <v>20</v>
+      </c>
+      <c r="D90" s="8">
+        <v>6</v>
+      </c>
+      <c r="E90" s="8">
+        <v>3</v>
+      </c>
+      <c r="F90" s="8">
+        <v>4</v>
+      </c>
       <c r="G90" s="8"/>
       <c r="H90" s="3"/>
       <c r="I90" s="3"/>
     </row>
     <row r="91" spans="1:9">
       <c r="A91" s="3"/>
-      <c r="B91" s="8"/>
-      <c r="C91" s="8"/>
-      <c r="D91" s="8"/>
-      <c r="E91" s="8"/>
-      <c r="F91" s="8"/>
+      <c r="B91" s="8">
+        <v>90</v>
+      </c>
+      <c r="C91" s="8">
+        <v>20</v>
+      </c>
+      <c r="D91" s="8">
+        <v>7</v>
+      </c>
+      <c r="E91" s="8">
+        <v>3</v>
+      </c>
+      <c r="F91" s="8">
+        <v>4</v>
+      </c>
       <c r="G91" s="8"/>
       <c r="H91" s="3"/>
       <c r="I91" s="3"/>
     </row>
     <row r="92" spans="1:9">
       <c r="A92" s="3"/>
-      <c r="B92" s="8"/>
-      <c r="C92" s="8"/>
-      <c r="D92" s="8"/>
-      <c r="E92" s="8"/>
-      <c r="F92" s="8"/>
+      <c r="B92" s="8">
+        <v>91</v>
+      </c>
+      <c r="C92" s="8">
+        <v>20</v>
+      </c>
+      <c r="D92" s="8">
+        <v>8</v>
+      </c>
+      <c r="E92" s="8">
+        <v>3</v>
+      </c>
+      <c r="F92" s="8">
+        <v>4</v>
+      </c>
       <c r="G92" s="8"/>
       <c r="H92" s="3"/>
       <c r="I92" s="3"/>
     </row>
     <row r="93" spans="1:9">
       <c r="A93" s="3"/>
-      <c r="B93" s="8"/>
-      <c r="C93" s="8"/>
-      <c r="D93" s="8"/>
-      <c r="E93" s="8"/>
-      <c r="F93" s="8"/>
+      <c r="B93" s="8">
+        <v>92</v>
+      </c>
+      <c r="C93" s="8">
+        <v>20</v>
+      </c>
+      <c r="D93" s="8">
+        <v>9</v>
+      </c>
+      <c r="E93" s="8">
+        <v>3</v>
+      </c>
+      <c r="F93" s="8">
+        <v>4</v>
+      </c>
       <c r="G93" s="8"/>
       <c r="H93" s="3"/>
       <c r="I93" s="3"/>
     </row>
     <row r="94" spans="1:9">
       <c r="A94" s="3"/>
-      <c r="B94" s="8"/>
-      <c r="C94" s="8"/>
-      <c r="D94" s="8"/>
-      <c r="E94" s="8"/>
-      <c r="F94" s="8"/>
+      <c r="B94" s="8">
+        <v>93</v>
+      </c>
+      <c r="C94" s="8">
+        <v>20</v>
+      </c>
+      <c r="D94" s="8">
+        <v>10</v>
+      </c>
+      <c r="E94" s="8">
+        <v>3</v>
+      </c>
+      <c r="F94" s="8">
+        <v>4</v>
+      </c>
       <c r="G94" s="8"/>
       <c r="H94" s="3"/>
       <c r="I94" s="3"/>
     </row>
     <row r="95" spans="1:9">
       <c r="A95" s="3"/>
-      <c r="B95" s="8"/>
-      <c r="C95" s="8"/>
-      <c r="D95" s="8"/>
-      <c r="E95" s="8"/>
-      <c r="F95" s="8"/>
+      <c r="B95" s="8">
+        <v>94</v>
+      </c>
+      <c r="C95" s="8">
+        <v>20</v>
+      </c>
+      <c r="D95" s="8">
+        <v>11</v>
+      </c>
+      <c r="E95" s="8">
+        <v>3</v>
+      </c>
+      <c r="F95" s="8">
+        <v>4</v>
+      </c>
       <c r="G95" s="8"/>
       <c r="H95" s="3"/>
       <c r="I95" s="3"/>
     </row>
     <row r="96" spans="1:9">
       <c r="A96" s="3"/>
-      <c r="B96" s="8"/>
-      <c r="C96" s="8"/>
-      <c r="D96" s="8"/>
-      <c r="E96" s="8"/>
-      <c r="F96" s="8"/>
+      <c r="B96" s="8">
+        <v>95</v>
+      </c>
+      <c r="C96" s="8">
+        <v>20</v>
+      </c>
+      <c r="D96" s="8">
+        <v>1</v>
+      </c>
+      <c r="E96" s="8">
+        <v>3</v>
+      </c>
+      <c r="F96" s="8">
+        <v>2.5</v>
+      </c>
       <c r="G96" s="8"/>
       <c r="H96" s="3"/>
       <c r="I96" s="3"/>
     </row>
     <row r="97" spans="1:9">
       <c r="A97" s="3"/>
-      <c r="B97" s="8"/>
-      <c r="C97" s="8"/>
-      <c r="D97" s="8"/>
-      <c r="E97" s="8"/>
-      <c r="F97" s="8"/>
+      <c r="B97" s="8">
+        <v>96</v>
+      </c>
+      <c r="C97" s="8">
+        <v>20</v>
+      </c>
+      <c r="D97" s="8">
+        <v>2</v>
+      </c>
+      <c r="E97" s="8">
+        <v>3</v>
+      </c>
+      <c r="F97" s="8">
+        <v>2.5</v>
+      </c>
       <c r="G97" s="8"/>
       <c r="H97" s="3"/>
       <c r="I97" s="3"/>
     </row>
     <row r="98" spans="1:9">
       <c r="A98" s="3"/>
-      <c r="B98" s="8"/>
-      <c r="C98" s="8"/>
-      <c r="D98" s="8"/>
-      <c r="E98" s="8"/>
-      <c r="F98" s="8"/>
+      <c r="B98" s="8">
+        <v>97</v>
+      </c>
+      <c r="C98" s="8">
+        <v>20</v>
+      </c>
+      <c r="D98" s="8">
+        <v>3</v>
+      </c>
+      <c r="E98" s="8">
+        <v>3</v>
+      </c>
+      <c r="F98" s="8">
+        <v>2.5</v>
+      </c>
       <c r="G98" s="8"/>
       <c r="H98" s="3"/>
       <c r="I98" s="3"/>
     </row>
     <row r="99" spans="1:9">
       <c r="A99" s="3"/>
-      <c r="B99" s="8"/>
-      <c r="C99" s="8"/>
-      <c r="D99" s="8"/>
-      <c r="E99" s="8"/>
-      <c r="F99" s="8"/>
+      <c r="B99" s="8">
+        <v>98</v>
+      </c>
+      <c r="C99" s="8">
+        <v>20</v>
+      </c>
+      <c r="D99" s="8">
+        <v>4</v>
+      </c>
+      <c r="E99" s="8">
+        <v>3</v>
+      </c>
+      <c r="F99" s="8">
+        <v>2.5</v>
+      </c>
       <c r="G99" s="8"/>
       <c r="H99" s="3"/>
       <c r="I99" s="3"/>
     </row>
     <row r="100" spans="1:9">
       <c r="A100" s="3"/>
-      <c r="B100" s="8"/>
-      <c r="C100" s="8"/>
-      <c r="D100" s="8"/>
-      <c r="E100" s="8"/>
-      <c r="F100" s="8"/>
+      <c r="B100" s="8">
+        <v>99</v>
+      </c>
+      <c r="C100" s="8">
+        <v>20</v>
+      </c>
+      <c r="D100" s="8">
+        <v>5</v>
+      </c>
+      <c r="E100" s="8">
+        <v>3</v>
+      </c>
+      <c r="F100" s="8">
+        <v>2.5</v>
+      </c>
       <c r="G100" s="8"/>
       <c r="H100" s="3"/>
       <c r="I100" s="3"/>
     </row>
     <row r="101" spans="1:9">
       <c r="A101" s="3"/>
-      <c r="B101" s="8"/>
-      <c r="C101" s="8"/>
-      <c r="D101" s="8"/>
-      <c r="E101" s="8"/>
-      <c r="F101" s="8"/>
+      <c r="B101" s="8">
+        <v>100</v>
+      </c>
+      <c r="C101" s="8">
+        <v>20</v>
+      </c>
+      <c r="D101" s="8">
+        <v>6</v>
+      </c>
+      <c r="E101" s="8">
+        <v>3</v>
+      </c>
+      <c r="F101" s="8">
+        <v>2.5</v>
+      </c>
       <c r="G101" s="8"/>
       <c r="H101" s="3"/>
       <c r="I101" s="3"/>
     </row>
     <row r="102" spans="1:9">
       <c r="A102" s="3"/>
-      <c r="B102" s="8"/>
-      <c r="C102" s="8"/>
-      <c r="D102" s="8"/>
-      <c r="E102" s="8"/>
-      <c r="F102" s="8"/>
+      <c r="B102" s="8">
+        <v>101</v>
+      </c>
+      <c r="C102" s="8">
+        <v>20</v>
+      </c>
+      <c r="D102" s="8">
+        <v>7</v>
+      </c>
+      <c r="E102" s="8">
+        <v>3</v>
+      </c>
+      <c r="F102" s="8">
+        <v>2.5</v>
+      </c>
       <c r="G102" s="8"/>
       <c r="H102" s="3"/>
       <c r="I102" s="3"/>
     </row>
     <row r="103" spans="1:9">
       <c r="A103" s="3"/>
-      <c r="B103" s="8"/>
-      <c r="C103" s="8"/>
-      <c r="D103" s="8"/>
-      <c r="E103" s="8"/>
-      <c r="F103" s="8"/>
+      <c r="B103" s="8">
+        <v>102</v>
+      </c>
+      <c r="C103" s="8">
+        <v>20</v>
+      </c>
+      <c r="D103" s="8">
+        <v>8</v>
+      </c>
+      <c r="E103" s="8">
+        <v>3</v>
+      </c>
+      <c r="F103" s="8">
+        <v>2.5</v>
+      </c>
       <c r="G103" s="8"/>
       <c r="H103" s="3"/>
       <c r="I103" s="3"/>
     </row>
     <row r="104" spans="1:9">
       <c r="A104" s="3"/>
-      <c r="B104" s="8"/>
-      <c r="C104" s="8"/>
-      <c r="D104" s="8"/>
-      <c r="E104" s="8"/>
-      <c r="F104" s="8"/>
+      <c r="B104" s="8">
+        <v>103</v>
+      </c>
+      <c r="C104" s="8">
+        <v>20</v>
+      </c>
+      <c r="D104" s="8">
+        <v>9</v>
+      </c>
+      <c r="E104" s="8">
+        <v>3</v>
+      </c>
+      <c r="F104" s="8">
+        <v>2.5</v>
+      </c>
       <c r="G104" s="8"/>
       <c r="H104" s="3"/>
       <c r="I104" s="3"/>
     </row>
     <row r="105" spans="1:9">
       <c r="A105" s="3"/>
-      <c r="B105" s="8"/>
-      <c r="C105" s="8"/>
-      <c r="D105" s="8"/>
-      <c r="E105" s="8"/>
-      <c r="F105" s="8"/>
+      <c r="B105" s="8">
+        <v>104</v>
+      </c>
+      <c r="C105" s="8">
+        <v>20</v>
+      </c>
+      <c r="D105" s="8">
+        <v>10</v>
+      </c>
+      <c r="E105" s="8">
+        <v>3</v>
+      </c>
+      <c r="F105" s="8">
+        <v>2.5</v>
+      </c>
       <c r="G105" s="8"/>
       <c r="H105" s="3"/>
       <c r="I105" s="3"/>
     </row>
     <row r="106" spans="1:9">
       <c r="A106" s="3"/>
-      <c r="B106" s="8"/>
-      <c r="C106" s="8"/>
-      <c r="D106" s="8"/>
-      <c r="E106" s="8"/>
-      <c r="F106" s="8"/>
+      <c r="B106" s="8">
+        <v>105</v>
+      </c>
+      <c r="C106" s="8">
+        <v>20</v>
+      </c>
+      <c r="D106" s="8">
+        <v>1</v>
+      </c>
+      <c r="E106" s="8">
+        <v>3</v>
+      </c>
+      <c r="F106" s="8">
+        <v>4.5</v>
+      </c>
       <c r="G106" s="8"/>
       <c r="H106" s="3"/>
       <c r="I106" s="3"/>
     </row>
     <row r="107" spans="1:9">
       <c r="A107" s="3"/>
-      <c r="B107" s="8"/>
-      <c r="C107" s="8"/>
-      <c r="D107" s="8"/>
-      <c r="E107" s="8"/>
-      <c r="F107" s="8"/>
+      <c r="B107" s="8">
+        <v>106</v>
+      </c>
+      <c r="C107" s="8">
+        <v>20</v>
+      </c>
+      <c r="D107" s="8">
+        <v>2</v>
+      </c>
+      <c r="E107" s="8">
+        <v>3</v>
+      </c>
+      <c r="F107" s="8">
+        <v>4.5</v>
+      </c>
       <c r="G107" s="8"/>
       <c r="H107" s="3"/>
       <c r="I107" s="3"/>
     </row>
     <row r="108" spans="1:9">
       <c r="A108" s="3"/>
-      <c r="B108" s="8"/>
-      <c r="C108" s="8"/>
-      <c r="D108" s="8"/>
-      <c r="E108" s="8"/>
-      <c r="F108" s="8"/>
+      <c r="B108" s="8">
+        <v>107</v>
+      </c>
+      <c r="C108" s="8">
+        <v>20</v>
+      </c>
+      <c r="D108" s="8">
+        <v>3</v>
+      </c>
+      <c r="E108" s="8">
+        <v>3</v>
+      </c>
+      <c r="F108" s="8">
+        <v>4.5</v>
+      </c>
       <c r="G108" s="8"/>
       <c r="H108" s="3"/>
       <c r="I108" s="3"/>
     </row>
     <row r="109" spans="1:9">
       <c r="A109" s="3"/>
-      <c r="B109" s="8"/>
-      <c r="C109" s="8"/>
-      <c r="D109" s="8"/>
-      <c r="E109" s="8"/>
-      <c r="F109" s="8"/>
+      <c r="B109" s="8">
+        <v>108</v>
+      </c>
+      <c r="C109" s="8">
+        <v>20</v>
+      </c>
+      <c r="D109" s="8">
+        <v>4</v>
+      </c>
+      <c r="E109" s="8">
+        <v>3</v>
+      </c>
+      <c r="F109" s="8">
+        <v>4.5</v>
+      </c>
       <c r="G109" s="8"/>
       <c r="H109" s="3"/>
       <c r="I109" s="3"/>
     </row>
     <row r="110" spans="1:9">
       <c r="A110" s="3"/>
-      <c r="B110" s="8"/>
-      <c r="C110" s="8"/>
-      <c r="D110" s="8"/>
-      <c r="E110" s="8"/>
-      <c r="F110" s="8"/>
+      <c r="B110" s="8">
+        <v>109</v>
+      </c>
+      <c r="C110" s="8">
+        <v>20</v>
+      </c>
+      <c r="D110" s="8">
+        <v>5</v>
+      </c>
+      <c r="E110" s="8">
+        <v>3</v>
+      </c>
+      <c r="F110" s="8">
+        <v>4.5</v>
+      </c>
       <c r="G110" s="8"/>
       <c r="H110" s="3"/>
       <c r="I110" s="3"/>
     </row>
     <row r="111" spans="1:9">
       <c r="A111" s="3"/>
-      <c r="B111" s="8"/>
-      <c r="C111" s="8"/>
-      <c r="D111" s="8"/>
-      <c r="E111" s="8"/>
-      <c r="F111" s="8"/>
+      <c r="B111" s="8">
+        <v>110</v>
+      </c>
+      <c r="C111" s="8">
+        <v>20</v>
+      </c>
+      <c r="D111" s="8">
+        <v>6</v>
+      </c>
+      <c r="E111" s="8">
+        <v>3</v>
+      </c>
+      <c r="F111" s="8">
+        <v>4.5</v>
+      </c>
       <c r="G111" s="8"/>
       <c r="H111" s="3"/>
       <c r="I111" s="3"/>
     </row>
     <row r="112" spans="1:9">
       <c r="A112" s="3"/>
-      <c r="B112" s="8"/>
-      <c r="C112" s="8"/>
-      <c r="D112" s="8"/>
-      <c r="E112" s="8"/>
-      <c r="F112" s="8"/>
+      <c r="B112" s="8">
+        <v>111</v>
+      </c>
+      <c r="C112" s="8">
+        <v>20</v>
+      </c>
+      <c r="D112" s="8">
+        <v>7</v>
+      </c>
+      <c r="E112" s="8">
+        <v>3</v>
+      </c>
+      <c r="F112" s="8">
+        <v>4.5</v>
+      </c>
       <c r="G112" s="8"/>
       <c r="H112" s="3"/>
       <c r="I112" s="3"/>
     </row>
     <row r="113" spans="1:9">
       <c r="A113" s="3"/>
-      <c r="B113" s="8"/>
-      <c r="C113" s="8"/>
-      <c r="D113" s="8"/>
-      <c r="E113" s="8"/>
-      <c r="F113" s="8"/>
+      <c r="B113" s="8">
+        <v>112</v>
+      </c>
+      <c r="C113" s="8">
+        <v>20</v>
+      </c>
+      <c r="D113" s="8">
+        <v>8</v>
+      </c>
+      <c r="E113" s="8">
+        <v>3</v>
+      </c>
+      <c r="F113" s="8">
+        <v>4.5</v>
+      </c>
       <c r="G113" s="8"/>
       <c r="H113" s="3"/>
       <c r="I113" s="3"/>
     </row>
     <row r="114" spans="1:9">
       <c r="A114" s="3"/>
-      <c r="B114" s="8"/>
-      <c r="C114" s="8"/>
-      <c r="D114" s="8"/>
-      <c r="E114" s="8"/>
-      <c r="F114" s="8"/>
+      <c r="B114" s="8">
+        <v>113</v>
+      </c>
+      <c r="C114" s="8">
+        <v>20</v>
+      </c>
+      <c r="D114" s="8">
+        <v>9</v>
+      </c>
+      <c r="E114" s="8">
+        <v>3</v>
+      </c>
+      <c r="F114" s="8">
+        <v>4.5</v>
+      </c>
       <c r="G114" s="8"/>
       <c r="H114" s="3"/>
       <c r="I114" s="3"/>
     </row>
     <row r="115" spans="1:9">
       <c r="A115" s="3"/>
-      <c r="B115" s="8"/>
-      <c r="C115" s="8"/>
-      <c r="D115" s="8"/>
-      <c r="E115" s="8"/>
-      <c r="F115" s="8"/>
+      <c r="B115" s="8">
+        <v>114</v>
+      </c>
+      <c r="C115" s="8">
+        <v>20</v>
+      </c>
+      <c r="D115" s="8">
+        <v>10</v>
+      </c>
+      <c r="E115" s="8">
+        <v>3</v>
+      </c>
+      <c r="F115" s="8">
+        <v>4.5</v>
+      </c>
       <c r="G115" s="8"/>
       <c r="H115" s="3"/>
       <c r="I115" s="3"/>
     </row>
     <row r="116" spans="1:9">
       <c r="A116" s="3"/>
-      <c r="B116" s="8"/>
-      <c r="C116" s="8"/>
-      <c r="D116" s="8"/>
-      <c r="E116" s="8"/>
-      <c r="F116" s="8"/>
+      <c r="B116" s="8">
+        <v>115</v>
+      </c>
+      <c r="C116" s="8">
+        <v>20</v>
+      </c>
+      <c r="D116" s="8">
+        <v>11</v>
+      </c>
+      <c r="E116" s="8">
+        <v>3</v>
+      </c>
+      <c r="F116" s="8">
+        <v>4.5</v>
+      </c>
       <c r="G116" s="8"/>
       <c r="H116" s="3"/>
       <c r="I116" s="3"/>
     </row>
     <row r="117" spans="1:9">
       <c r="A117" s="3"/>
-      <c r="B117" s="8"/>
-      <c r="C117" s="8"/>
-      <c r="D117" s="8"/>
-      <c r="E117" s="8"/>
-      <c r="F117" s="8"/>
+      <c r="B117" s="8">
+        <v>116</v>
+      </c>
+      <c r="C117" s="8">
+        <v>20</v>
+      </c>
+      <c r="D117" s="8">
+        <v>12</v>
+      </c>
+      <c r="E117" s="8">
+        <v>3</v>
+      </c>
+      <c r="F117" s="8">
+        <v>4.5</v>
+      </c>
       <c r="G117" s="8"/>
       <c r="H117" s="3"/>
       <c r="I117" s="3"/>
     </row>
     <row r="118" spans="1:9">
       <c r="A118" s="3"/>
-      <c r="B118" s="8"/>
-      <c r="C118" s="8"/>
-      <c r="D118" s="8"/>
-      <c r="E118" s="8"/>
-      <c r="F118" s="8"/>
+      <c r="B118" s="8">
+        <v>117</v>
+      </c>
+      <c r="C118" s="8">
+        <v>20</v>
+      </c>
+      <c r="D118" s="8">
+        <v>12</v>
+      </c>
+      <c r="E118" s="8">
+        <v>3</v>
+      </c>
+      <c r="F118" s="8">
+        <v>5</v>
+      </c>
       <c r="G118" s="8"/>
       <c r="H118" s="3"/>
       <c r="I118" s="3"/>
     </row>
     <row r="119" spans="1:9">
       <c r="A119" s="3"/>
-      <c r="B119" s="8"/>
-      <c r="C119" s="8"/>
-      <c r="D119" s="8"/>
-      <c r="E119" s="8"/>
-      <c r="F119" s="8"/>
+      <c r="B119" s="8">
+        <v>118</v>
+      </c>
+      <c r="C119" s="8">
+        <v>20</v>
+      </c>
+      <c r="D119" s="8">
+        <v>11</v>
+      </c>
+      <c r="E119" s="8">
+        <v>3</v>
+      </c>
+      <c r="F119" s="8">
+        <v>5</v>
+      </c>
       <c r="G119" s="8"/>
       <c r="H119" s="3"/>
       <c r="I119" s="3"/>
     </row>
     <row r="120" spans="1:9">
       <c r="A120" s="3"/>
-      <c r="B120" s="8"/>
-      <c r="C120" s="8"/>
-      <c r="D120" s="8"/>
-      <c r="E120" s="8"/>
-      <c r="F120" s="8"/>
+      <c r="B120" s="8">
+        <v>119</v>
+      </c>
+      <c r="C120" s="8">
+        <v>20</v>
+      </c>
+      <c r="D120" s="8">
+        <v>10</v>
+      </c>
+      <c r="E120" s="8">
+        <v>3</v>
+      </c>
+      <c r="F120" s="8">
+        <v>5</v>
+      </c>
       <c r="G120" s="8"/>
       <c r="H120" s="3"/>
       <c r="I120" s="3"/>
     </row>
     <row r="121" spans="1:9">
       <c r="A121" s="3"/>
-      <c r="B121" s="8"/>
-      <c r="C121" s="8"/>
-      <c r="D121" s="8"/>
-      <c r="E121" s="8"/>
-      <c r="F121" s="8"/>
+      <c r="B121" s="8">
+        <v>120</v>
+      </c>
+      <c r="C121" s="8">
+        <v>20</v>
+      </c>
+      <c r="D121" s="8">
+        <v>9</v>
+      </c>
+      <c r="E121" s="8">
+        <v>3</v>
+      </c>
+      <c r="F121" s="8">
+        <v>5</v>
+      </c>
       <c r="G121" s="8"/>
       <c r="H121" s="3"/>
       <c r="I121" s="3"/>
     </row>
     <row r="122" spans="1:9">
       <c r="A122" s="3"/>
-      <c r="B122" s="8"/>
-      <c r="C122" s="8"/>
-      <c r="D122" s="8"/>
-      <c r="E122" s="8"/>
-      <c r="F122" s="8"/>
+      <c r="B122" s="8">
+        <v>121</v>
+      </c>
+      <c r="C122" s="8">
+        <v>20</v>
+      </c>
+      <c r="D122" s="8">
+        <v>8</v>
+      </c>
+      <c r="E122" s="8">
+        <v>3</v>
+      </c>
+      <c r="F122" s="8">
+        <v>5</v>
+      </c>
       <c r="G122" s="8"/>
       <c r="H122" s="3"/>
       <c r="I122" s="3"/>
     </row>
     <row r="123" spans="1:9">
       <c r="A123" s="3"/>
-      <c r="B123" s="8"/>
-      <c r="C123" s="8"/>
-      <c r="D123" s="8"/>
-      <c r="E123" s="8"/>
-      <c r="F123" s="8"/>
+      <c r="B123" s="8">
+        <v>122</v>
+      </c>
+      <c r="C123" s="8">
+        <v>20</v>
+      </c>
+      <c r="D123" s="8">
+        <v>7</v>
+      </c>
+      <c r="E123" s="8">
+        <v>3</v>
+      </c>
+      <c r="F123" s="8">
+        <v>5</v>
+      </c>
       <c r="G123" s="8"/>
       <c r="H123" s="3"/>
       <c r="I123" s="3"/>
     </row>
-    <row r="124" spans="1:9">
+    <row r="124" ht="14.4" spans="1:9">
       <c r="A124" s="3"/>
-      <c r="B124" s="8"/>
-      <c r="C124" s="8"/>
-      <c r="D124" s="8"/>
-      <c r="E124" s="8"/>
-      <c r="F124" s="8"/>
+      <c r="B124" s="8">
+        <v>123</v>
+      </c>
+      <c r="C124" s="8">
+        <v>10</v>
+      </c>
+      <c r="D124" s="8">
+        <v>6</v>
+      </c>
+      <c r="E124" s="8">
+        <v>3</v>
+      </c>
+      <c r="F124" s="8">
+        <v>5</v>
+      </c>
       <c r="G124" s="8"/>
       <c r="H124" s="3"/>
-      <c r="I124" s="3"/>
+      <c r="I124" s="9" t="s">
+        <v>22</v>
+      </c>
     </row>
     <row r="125" spans="1:9">
       <c r="A125" s="3"/>
-      <c r="B125" s="8"/>
-      <c r="C125" s="8"/>
-      <c r="D125" s="8"/>
-      <c r="E125" s="8"/>
-      <c r="F125" s="8"/>
+      <c r="B125" s="8">
+        <v>124</v>
+      </c>
+      <c r="C125" s="8">
+        <v>10</v>
+      </c>
+      <c r="D125" s="8">
+        <v>5</v>
+      </c>
+      <c r="E125" s="8">
+        <v>3</v>
+      </c>
+      <c r="F125" s="8">
+        <v>5</v>
+      </c>
       <c r="G125" s="8"/>
       <c r="H125" s="3"/>
       <c r="I125" s="3"/>
     </row>
     <row r="126" spans="1:9">
       <c r="A126" s="3"/>
-      <c r="B126" s="8"/>
-      <c r="C126" s="8"/>
-      <c r="D126" s="8"/>
-      <c r="E126" s="8"/>
-      <c r="F126" s="8"/>
+      <c r="B126" s="8">
+        <v>125</v>
+      </c>
+      <c r="C126" s="8">
+        <v>10</v>
+      </c>
+      <c r="D126" s="8">
+        <v>4</v>
+      </c>
+      <c r="E126" s="8">
+        <v>3</v>
+      </c>
+      <c r="F126" s="8">
+        <v>5</v>
+      </c>
       <c r="G126" s="8"/>
       <c r="H126" s="3"/>
       <c r="I126" s="3"/>
     </row>
     <row r="127" spans="1:9">
       <c r="A127" s="3"/>
-      <c r="B127" s="8"/>
-      <c r="C127" s="8"/>
-      <c r="D127" s="8"/>
-      <c r="E127" s="8"/>
-      <c r="F127" s="8"/>
+      <c r="B127" s="8">
+        <v>126</v>
+      </c>
+      <c r="C127" s="8">
+        <v>10</v>
+      </c>
+      <c r="D127" s="8">
+        <v>3</v>
+      </c>
+      <c r="E127" s="8">
+        <v>3</v>
+      </c>
+      <c r="F127" s="8">
+        <v>5</v>
+      </c>
       <c r="G127" s="8"/>
       <c r="H127" s="3"/>
       <c r="I127" s="3"/>
     </row>
     <row r="128" spans="1:9">
       <c r="A128" s="3"/>
-      <c r="B128" s="8"/>
-      <c r="C128" s="8"/>
-      <c r="D128" s="8"/>
-      <c r="E128" s="8"/>
-      <c r="F128" s="8"/>
+      <c r="B128" s="8">
+        <v>127</v>
+      </c>
+      <c r="C128" s="8">
+        <v>10</v>
+      </c>
+      <c r="D128" s="8">
+        <v>2</v>
+      </c>
+      <c r="E128" s="8">
+        <v>3</v>
+      </c>
+      <c r="F128" s="8">
+        <v>5</v>
+      </c>
       <c r="G128" s="8"/>
       <c r="H128" s="3"/>
       <c r="I128" s="3"/>
     </row>
-    <row r="129" spans="1:9">
+    <row r="129" ht="14.4" spans="1:9">
       <c r="A129" s="3"/>
-      <c r="B129" s="8"/>
-      <c r="C129" s="8"/>
-      <c r="D129" s="8"/>
-      <c r="E129" s="8"/>
-      <c r="F129" s="8"/>
+      <c r="B129" s="8">
+        <v>128</v>
+      </c>
+      <c r="C129" s="8">
+        <v>20</v>
+      </c>
+      <c r="D129" s="8">
+        <v>6</v>
+      </c>
+      <c r="E129" s="8">
+        <v>3</v>
+      </c>
+      <c r="F129" s="8">
+        <v>5</v>
+      </c>
       <c r="G129" s="8"/>
       <c r="H129" s="3"/>
-      <c r="I129" s="3"/>
+      <c r="I129" s="9" t="s">
+        <v>23</v>
+      </c>
     </row>
     <row r="130" spans="1:9">
       <c r="A130" s="3"/>
-      <c r="B130" s="8"/>
-      <c r="C130" s="8"/>
-      <c r="D130" s="8"/>
-      <c r="E130" s="8"/>
-      <c r="F130" s="8"/>
+      <c r="B130" s="8">
+        <v>129</v>
+      </c>
+      <c r="C130" s="8">
+        <v>20</v>
+      </c>
+      <c r="D130" s="8">
+        <v>5</v>
+      </c>
+      <c r="E130" s="8">
+        <v>3</v>
+      </c>
+      <c r="F130" s="8">
+        <v>5</v>
+      </c>
       <c r="G130" s="8"/>
       <c r="H130" s="3"/>
       <c r="I130" s="3"/>
     </row>
     <row r="131" spans="1:9">
       <c r="A131" s="3"/>
-      <c r="B131" s="8"/>
-      <c r="C131" s="8"/>
-      <c r="D131" s="8"/>
-      <c r="E131" s="8"/>
-      <c r="F131" s="8"/>
+      <c r="B131" s="8">
+        <v>130</v>
+      </c>
+      <c r="C131" s="8">
+        <v>20</v>
+      </c>
+      <c r="D131" s="8">
+        <v>4</v>
+      </c>
+      <c r="E131" s="8">
+        <v>3</v>
+      </c>
+      <c r="F131" s="8">
+        <v>5</v>
+      </c>
       <c r="G131" s="8"/>
       <c r="H131" s="3"/>
       <c r="I131" s="3"/>
     </row>
     <row r="132" spans="1:9">
       <c r="A132" s="3"/>
-      <c r="B132" s="8"/>
-      <c r="C132" s="8"/>
-      <c r="D132" s="8"/>
-      <c r="E132" s="8"/>
-      <c r="F132" s="8"/>
+      <c r="B132" s="8">
+        <v>131</v>
+      </c>
+      <c r="C132" s="8">
+        <v>20</v>
+      </c>
+      <c r="D132" s="8">
+        <v>3</v>
+      </c>
+      <c r="E132" s="8">
+        <v>3</v>
+      </c>
+      <c r="F132" s="8">
+        <v>5</v>
+      </c>
       <c r="G132" s="8"/>
       <c r="H132" s="3"/>
       <c r="I132" s="3"/>
     </row>
     <row r="133" spans="1:9">
       <c r="A133" s="3"/>
-      <c r="B133" s="8"/>
-      <c r="C133" s="8"/>
-      <c r="D133" s="8"/>
-      <c r="E133" s="8"/>
-      <c r="F133" s="8"/>
+      <c r="B133" s="8">
+        <v>132</v>
+      </c>
+      <c r="C133" s="8">
+        <v>10</v>
+      </c>
+      <c r="D133" s="8">
+        <v>7</v>
+      </c>
+      <c r="E133" s="8">
+        <v>3</v>
+      </c>
+      <c r="F133" s="8">
+        <v>5</v>
+      </c>
       <c r="G133" s="8"/>
       <c r="H133" s="3"/>
       <c r="I133" s="3"/>
     </row>
     <row r="134" spans="1:9">
       <c r="A134" s="3"/>
-      <c r="B134" s="8"/>
-      <c r="C134" s="8"/>
-      <c r="D134" s="8"/>
-      <c r="E134" s="8"/>
-      <c r="F134" s="8"/>
+      <c r="B134" s="8">
+        <v>133</v>
+      </c>
+      <c r="C134" s="8">
+        <v>10</v>
+      </c>
+      <c r="D134" s="8">
+        <v>8</v>
+      </c>
+      <c r="E134" s="8">
+        <v>3</v>
+      </c>
+      <c r="F134" s="8">
+        <v>5</v>
+      </c>
       <c r="G134" s="8"/>
       <c r="H134" s="3"/>
       <c r="I134" s="3"/>
     </row>
     <row r="135" spans="1:9">
       <c r="A135" s="3"/>
-      <c r="B135" s="8"/>
-      <c r="C135" s="8"/>
-      <c r="D135" s="8"/>
-      <c r="E135" s="8"/>
-      <c r="F135" s="8"/>
+      <c r="B135" s="8">
+        <v>134</v>
+      </c>
+      <c r="C135" s="8">
+        <v>10</v>
+      </c>
+      <c r="D135" s="8">
+        <v>8</v>
+      </c>
+      <c r="E135" s="8">
+        <v>3</v>
+      </c>
+      <c r="F135" s="8">
+        <v>4.5</v>
+      </c>
       <c r="G135" s="8"/>
       <c r="H135" s="3"/>
       <c r="I135" s="3"/>
     </row>
     <row r="136" spans="1:9">
       <c r="A136" s="3"/>
-      <c r="B136" s="8"/>
-      <c r="C136" s="8"/>
-      <c r="D136" s="8"/>
-      <c r="E136" s="8"/>
-      <c r="F136" s="8"/>
+      <c r="B136" s="8">
+        <v>135</v>
+      </c>
+      <c r="C136" s="8">
+        <v>10</v>
+      </c>
+      <c r="D136" s="8">
+        <v>7</v>
+      </c>
+      <c r="E136" s="8">
+        <v>3</v>
+      </c>
+      <c r="F136" s="8">
+        <v>4.5</v>
+      </c>
       <c r="G136" s="8"/>
       <c r="H136" s="3"/>
       <c r="I136" s="3"/>
     </row>
     <row r="137" spans="1:9">
       <c r="A137" s="3"/>
-      <c r="B137" s="8"/>
-      <c r="C137" s="8"/>
-      <c r="D137" s="8"/>
-      <c r="E137" s="8"/>
-      <c r="F137" s="8"/>
+      <c r="B137" s="8">
+        <v>136</v>
+      </c>
+      <c r="C137" s="8">
+        <v>10</v>
+      </c>
+      <c r="D137" s="8">
+        <v>6</v>
+      </c>
+      <c r="E137" s="8">
+        <v>3</v>
+      </c>
+      <c r="F137" s="8">
+        <v>4.5</v>
+      </c>
       <c r="G137" s="8"/>
       <c r="H137" s="3"/>
       <c r="I137" s="3"/>
     </row>
     <row r="138" spans="1:9">
       <c r="A138" s="3"/>
-      <c r="B138" s="8"/>
-      <c r="C138" s="8"/>
-      <c r="D138" s="8"/>
-      <c r="E138" s="8"/>
-      <c r="F138" s="8"/>
+      <c r="B138" s="8">
+        <v>137</v>
+      </c>
+      <c r="C138" s="8">
+        <v>10</v>
+      </c>
+      <c r="D138" s="8">
+        <v>5</v>
+      </c>
+      <c r="E138" s="8">
+        <v>3</v>
+      </c>
+      <c r="F138" s="8">
+        <v>4.5</v>
+      </c>
       <c r="G138" s="8"/>
       <c r="H138" s="3"/>
       <c r="I138" s="3"/>
     </row>
     <row r="139" spans="1:9">
       <c r="A139" s="3"/>
-      <c r="B139" s="8"/>
-      <c r="C139" s="8"/>
-      <c r="D139" s="8"/>
-      <c r="E139" s="8"/>
-      <c r="F139" s="8"/>
+      <c r="B139" s="8">
+        <v>138</v>
+      </c>
+      <c r="C139" s="8">
+        <v>10</v>
+      </c>
+      <c r="D139" s="8">
+        <v>4</v>
+      </c>
+      <c r="E139" s="8">
+        <v>3</v>
+      </c>
+      <c r="F139" s="8">
+        <v>4.5</v>
+      </c>
       <c r="G139" s="8"/>
       <c r="H139" s="3"/>
       <c r="I139" s="3"/>
     </row>
     <row r="140" spans="1:9">
       <c r="A140" s="3"/>
-      <c r="B140" s="8"/>
-      <c r="C140" s="8"/>
-      <c r="D140" s="8"/>
-      <c r="E140" s="8"/>
-      <c r="F140" s="8"/>
+      <c r="B140" s="8">
+        <v>139</v>
+      </c>
+      <c r="C140" s="8">
+        <v>10</v>
+      </c>
+      <c r="D140" s="8">
+        <v>3</v>
+      </c>
+      <c r="E140" s="8">
+        <v>3</v>
+      </c>
+      <c r="F140" s="8">
+        <v>4.5</v>
+      </c>
       <c r="G140" s="8"/>
       <c r="H140" s="3"/>
       <c r="I140" s="3"/>
     </row>
     <row r="141" spans="1:9">
       <c r="A141" s="3"/>
-      <c r="B141" s="8"/>
-      <c r="C141" s="8"/>
-      <c r="D141" s="8"/>
-      <c r="E141" s="8"/>
-      <c r="F141" s="8"/>
+      <c r="B141" s="8">
+        <v>140</v>
+      </c>
+      <c r="C141" s="8">
+        <v>10</v>
+      </c>
+      <c r="D141" s="8">
+        <v>2</v>
+      </c>
+      <c r="E141" s="8">
+        <v>3</v>
+      </c>
+      <c r="F141" s="8">
+        <v>4.5</v>
+      </c>
       <c r="G141" s="8"/>
       <c r="H141" s="3"/>
       <c r="I141" s="3"/>
     </row>
     <row r="142" spans="1:9">
       <c r="A142" s="3"/>
-      <c r="B142" s="8"/>
-      <c r="C142" s="8"/>
-      <c r="D142" s="8"/>
-      <c r="E142" s="8"/>
-      <c r="F142" s="8"/>
+      <c r="B142" s="8">
+        <v>141</v>
+      </c>
+      <c r="C142" s="8">
+        <v>10</v>
+      </c>
+      <c r="D142" s="8">
+        <v>8</v>
+      </c>
+      <c r="E142" s="8">
+        <v>3</v>
+      </c>
+      <c r="F142" s="8">
+        <v>4</v>
+      </c>
       <c r="G142" s="8"/>
       <c r="H142" s="3"/>
       <c r="I142" s="3"/>
     </row>
     <row r="143" spans="1:9">
       <c r="A143" s="3"/>
-      <c r="B143" s="8"/>
-      <c r="C143" s="8"/>
-      <c r="D143" s="8"/>
-      <c r="E143" s="8"/>
-      <c r="F143" s="8"/>
+      <c r="B143" s="8">
+        <v>142</v>
+      </c>
+      <c r="C143" s="8">
+        <v>10</v>
+      </c>
+      <c r="D143" s="8">
+        <v>7</v>
+      </c>
+      <c r="E143" s="8">
+        <v>3</v>
+      </c>
+      <c r="F143" s="8">
+        <v>4</v>
+      </c>
       <c r="G143" s="8"/>
       <c r="H143" s="3"/>
       <c r="I143" s="3"/>
     </row>
     <row r="144" spans="1:9">
       <c r="A144" s="3"/>
-      <c r="B144" s="8"/>
-      <c r="C144" s="8"/>
-      <c r="D144" s="8"/>
-      <c r="E144" s="8"/>
-      <c r="F144" s="8"/>
+      <c r="B144" s="8">
+        <v>143</v>
+      </c>
+      <c r="C144" s="8">
+        <v>10</v>
+      </c>
+      <c r="D144" s="8">
+        <v>6</v>
+      </c>
+      <c r="E144" s="8">
+        <v>3</v>
+      </c>
+      <c r="F144" s="8">
+        <v>4</v>
+      </c>
       <c r="G144" s="8"/>
       <c r="H144" s="3"/>
       <c r="I144" s="3"/>
     </row>
     <row r="145" spans="1:9">
       <c r="A145" s="3"/>
-      <c r="B145" s="8"/>
-      <c r="C145" s="8"/>
-      <c r="D145" s="8"/>
-      <c r="E145" s="8"/>
-      <c r="F145" s="8"/>
+      <c r="B145" s="8">
+        <v>144</v>
+      </c>
+      <c r="C145" s="8">
+        <v>10</v>
+      </c>
+      <c r="D145" s="8">
+        <v>5</v>
+      </c>
+      <c r="E145" s="8">
+        <v>3</v>
+      </c>
+      <c r="F145" s="8">
+        <v>4</v>
+      </c>
       <c r="G145" s="8"/>
       <c r="H145" s="3"/>
       <c r="I145" s="3"/>
     </row>
     <row r="146" spans="1:9">
       <c r="A146" s="3"/>
-      <c r="B146" s="8"/>
-      <c r="C146" s="8"/>
-      <c r="D146" s="8"/>
-      <c r="E146" s="8"/>
-      <c r="F146" s="8"/>
+      <c r="B146" s="8">
+        <v>145</v>
+      </c>
+      <c r="C146" s="8">
+        <v>10</v>
+      </c>
+      <c r="D146" s="8">
+        <v>4</v>
+      </c>
+      <c r="E146" s="8">
+        <v>3</v>
+      </c>
+      <c r="F146" s="8">
+        <v>4</v>
+      </c>
       <c r="G146" s="8"/>
       <c r="H146" s="3"/>
       <c r="I146" s="3"/>
     </row>
     <row r="147" spans="1:9">
       <c r="A147" s="3"/>
-      <c r="B147" s="8"/>
-      <c r="C147" s="8"/>
-      <c r="D147" s="8"/>
-      <c r="E147" s="8"/>
-      <c r="F147" s="8"/>
+      <c r="B147" s="8">
+        <v>146</v>
+      </c>
+      <c r="C147" s="8">
+        <v>10</v>
+      </c>
+      <c r="D147" s="8">
+        <v>3</v>
+      </c>
+      <c r="E147" s="8">
+        <v>3</v>
+      </c>
+      <c r="F147" s="8">
+        <v>4</v>
+      </c>
       <c r="G147" s="8"/>
       <c r="H147" s="3"/>
       <c r="I147" s="3"/>
     </row>
     <row r="148" spans="1:9">
       <c r="A148" s="3"/>
-      <c r="B148" s="8"/>
-      <c r="C148" s="8"/>
-      <c r="D148" s="8"/>
-      <c r="E148" s="8"/>
-      <c r="F148" s="8"/>
+      <c r="B148" s="8">
+        <v>147</v>
+      </c>
+      <c r="C148" s="8">
+        <v>10</v>
+      </c>
+      <c r="D148" s="8">
+        <v>2</v>
+      </c>
+      <c r="E148" s="8">
+        <v>3</v>
+      </c>
+      <c r="F148" s="8">
+        <v>4</v>
+      </c>
       <c r="G148" s="8"/>
       <c r="H148" s="3"/>
       <c r="I148" s="3"/>
     </row>
     <row r="149" spans="1:9">
       <c r="A149" s="3"/>
-      <c r="B149" s="8"/>
-      <c r="C149" s="8"/>
-      <c r="D149" s="8"/>
-      <c r="E149" s="8"/>
-      <c r="F149" s="8"/>
+      <c r="B149" s="8">
+        <v>148</v>
+      </c>
+      <c r="C149" s="8">
+        <v>10</v>
+      </c>
+      <c r="D149" s="8">
+        <v>1</v>
+      </c>
+      <c r="E149" s="8">
+        <v>3</v>
+      </c>
+      <c r="F149" s="8">
+        <v>4</v>
+      </c>
       <c r="G149" s="8"/>
       <c r="H149" s="3"/>
       <c r="I149" s="3"/>
     </row>
     <row r="150" spans="1:9">
       <c r="A150" s="3"/>
-      <c r="B150" s="8"/>
-      <c r="C150" s="8"/>
-      <c r="D150" s="8"/>
-      <c r="E150" s="8"/>
-      <c r="F150" s="8"/>
+      <c r="B150" s="8">
+        <v>149</v>
+      </c>
+      <c r="C150" s="8">
+        <v>10</v>
+      </c>
+      <c r="D150" s="8">
+        <v>8</v>
+      </c>
+      <c r="E150" s="8">
+        <v>3</v>
+      </c>
+      <c r="F150" s="8">
+        <v>3.5</v>
+      </c>
       <c r="G150" s="8"/>
       <c r="H150" s="3"/>
       <c r="I150" s="3"/>
     </row>
     <row r="151" spans="1:9">
       <c r="A151" s="3"/>
-      <c r="B151" s="8"/>
-      <c r="C151" s="8"/>
-      <c r="D151" s="8"/>
-      <c r="E151" s="8"/>
-      <c r="F151" s="8"/>
+      <c r="B151" s="8">
+        <v>150</v>
+      </c>
+      <c r="C151" s="8">
+        <v>10</v>
+      </c>
+      <c r="D151" s="8">
+        <v>7</v>
+      </c>
+      <c r="E151" s="8">
+        <v>3</v>
+      </c>
+      <c r="F151" s="8">
+        <v>3.5</v>
+      </c>
       <c r="G151" s="8"/>
       <c r="H151" s="3"/>
       <c r="I151" s="3"/>
     </row>
     <row r="152" spans="1:9">
       <c r="A152" s="3"/>
-      <c r="B152" s="8"/>
-      <c r="C152" s="8"/>
-      <c r="D152" s="8"/>
-      <c r="E152" s="8"/>
-      <c r="F152" s="8"/>
+      <c r="B152" s="8">
+        <v>151</v>
+      </c>
+      <c r="C152" s="8">
+        <v>10</v>
+      </c>
+      <c r="D152" s="8">
+        <v>6</v>
+      </c>
+      <c r="E152" s="8">
+        <v>3</v>
+      </c>
+      <c r="F152" s="8">
+        <v>3.5</v>
+      </c>
       <c r="G152" s="8"/>
       <c r="H152" s="3"/>
       <c r="I152" s="3"/>
     </row>
     <row r="153" spans="1:9">
       <c r="A153" s="3"/>
-      <c r="B153" s="8"/>
-      <c r="C153" s="8"/>
-      <c r="D153" s="8"/>
-      <c r="E153" s="8"/>
-      <c r="F153" s="8"/>
+      <c r="B153" s="8">
+        <v>152</v>
+      </c>
+      <c r="C153" s="8">
+        <v>10</v>
+      </c>
+      <c r="D153" s="8">
+        <v>5</v>
+      </c>
+      <c r="E153" s="8">
+        <v>3</v>
+      </c>
+      <c r="F153" s="8">
+        <v>3.5</v>
+      </c>
       <c r="G153" s="8"/>
       <c r="H153" s="3"/>
       <c r="I153" s="3"/>
     </row>
     <row r="154" spans="1:9">
       <c r="A154" s="3"/>
-      <c r="B154" s="8"/>
-      <c r="C154" s="8"/>
-      <c r="D154" s="8"/>
-      <c r="E154" s="8"/>
-      <c r="F154" s="8"/>
+      <c r="B154" s="8">
+        <v>153</v>
+      </c>
+      <c r="C154" s="8">
+        <v>10</v>
+      </c>
+      <c r="D154" s="8">
+        <v>4</v>
+      </c>
+      <c r="E154" s="8">
+        <v>3</v>
+      </c>
+      <c r="F154" s="8">
+        <v>3.5</v>
+      </c>
       <c r="G154" s="8"/>
       <c r="H154" s="3"/>
       <c r="I154" s="3"/>
     </row>
     <row r="155" spans="1:9">
       <c r="A155" s="3"/>
-      <c r="B155" s="8"/>
-      <c r="C155" s="8"/>
-      <c r="D155" s="8"/>
-      <c r="E155" s="8"/>
-      <c r="F155" s="8"/>
+      <c r="B155" s="8">
+        <v>154</v>
+      </c>
+      <c r="C155" s="8">
+        <v>10</v>
+      </c>
+      <c r="D155" s="8">
+        <v>3</v>
+      </c>
+      <c r="E155" s="8">
+        <v>3</v>
+      </c>
+      <c r="F155" s="8">
+        <v>3.5</v>
+      </c>
       <c r="G155" s="8"/>
       <c r="H155" s="3"/>
       <c r="I155" s="3"/>
     </row>
     <row r="156" spans="1:9">
       <c r="A156" s="3"/>
-      <c r="B156" s="8"/>
-      <c r="C156" s="8"/>
-      <c r="D156" s="8"/>
-      <c r="E156" s="8"/>
-      <c r="F156" s="8"/>
+      <c r="B156" s="8">
+        <v>155</v>
+      </c>
+      <c r="C156" s="8">
+        <v>10</v>
+      </c>
+      <c r="D156" s="8">
+        <v>2</v>
+      </c>
+      <c r="E156" s="8">
+        <v>3</v>
+      </c>
+      <c r="F156" s="8">
+        <v>3.5</v>
+      </c>
       <c r="G156" s="8"/>
       <c r="H156" s="3"/>
       <c r="I156" s="3"/>
     </row>
     <row r="157" spans="1:9">
       <c r="A157" s="3"/>
-      <c r="B157" s="8"/>
-      <c r="C157" s="8"/>
-      <c r="D157" s="8"/>
-      <c r="E157" s="8"/>
-      <c r="F157" s="8"/>
+      <c r="B157" s="8">
+        <v>156</v>
+      </c>
+      <c r="C157" s="8">
+        <v>10</v>
+      </c>
+      <c r="D157" s="8">
+        <v>1</v>
+      </c>
+      <c r="E157" s="8">
+        <v>3</v>
+      </c>
+      <c r="F157" s="8">
+        <v>3.5</v>
+      </c>
       <c r="G157" s="8"/>
       <c r="H157" s="3"/>
       <c r="I157" s="3"/>
     </row>
     <row r="158" spans="1:9">
       <c r="A158" s="3"/>
-      <c r="B158" s="8"/>
-      <c r="C158" s="8"/>
-      <c r="D158" s="8"/>
-      <c r="E158" s="8"/>
-      <c r="F158" s="8"/>
+      <c r="B158" s="8">
+        <v>157</v>
+      </c>
+      <c r="C158" s="8">
+        <v>10</v>
+      </c>
+      <c r="D158" s="8">
+        <v>1</v>
+      </c>
+      <c r="E158" s="8">
+        <v>3</v>
+      </c>
+      <c r="F158" s="8">
+        <v>3</v>
+      </c>
       <c r="G158" s="8"/>
       <c r="H158" s="3"/>
       <c r="I158" s="3"/>
     </row>
     <row r="159" spans="1:9">
       <c r="A159" s="3"/>
-      <c r="B159" s="8"/>
-      <c r="C159" s="8"/>
-      <c r="D159" s="8"/>
-      <c r="E159" s="8"/>
-      <c r="F159" s="8"/>
+      <c r="B159" s="8">
+        <v>158</v>
+      </c>
+      <c r="C159" s="8">
+        <v>10</v>
+      </c>
+      <c r="D159" s="8">
+        <v>2</v>
+      </c>
+      <c r="E159" s="8">
+        <v>3</v>
+      </c>
+      <c r="F159" s="8">
+        <v>3</v>
+      </c>
       <c r="G159" s="8"/>
       <c r="H159" s="3"/>
       <c r="I159" s="3"/>
     </row>
     <row r="160" spans="1:9">
       <c r="A160" s="3"/>
-      <c r="B160" s="8"/>
-      <c r="C160" s="8"/>
-      <c r="D160" s="8"/>
-      <c r="E160" s="8"/>
-      <c r="F160" s="8"/>
+      <c r="B160" s="8">
+        <v>159</v>
+      </c>
+      <c r="C160" s="8">
+        <v>10</v>
+      </c>
+      <c r="D160" s="8">
+        <v>3</v>
+      </c>
+      <c r="E160" s="8">
+        <v>3</v>
+      </c>
+      <c r="F160" s="8">
+        <v>3</v>
+      </c>
       <c r="G160" s="8"/>
       <c r="H160" s="3"/>
       <c r="I160" s="3"/>
     </row>
     <row r="161" spans="1:9">
       <c r="A161" s="3"/>
-      <c r="B161" s="8"/>
-      <c r="C161" s="8"/>
-      <c r="D161" s="8"/>
-      <c r="E161" s="8"/>
-      <c r="F161" s="8"/>
+      <c r="B161" s="8">
+        <v>160</v>
+      </c>
+      <c r="C161" s="8">
+        <v>10</v>
+      </c>
+      <c r="D161" s="8">
+        <v>4</v>
+      </c>
+      <c r="E161" s="8">
+        <v>3</v>
+      </c>
+      <c r="F161" s="8">
+        <v>3</v>
+      </c>
       <c r="G161" s="8"/>
       <c r="H161" s="3"/>
       <c r="I161" s="3"/>

</xml_diff>